<commit_message>
fix: corregir mensajes de validación en Excel y sincronizar con la web
</commit_message>
<xml_diff>
--- a/src/test/java/org/utils/Registros.xlsx
+++ b/src/test/java/org/utils/Registros.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\IdeaProjects\MiBilleteraAT\src\test\java\org\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3132A3A8-798A-4C5B-8871-3BECA4EA10F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62DD8091-B4B0-4300-973B-1803975E03A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D4E4FA09-44F9-4DC2-A071-5AAC37EF05C6}"/>
   </bookViews>
@@ -84,18 +84,12 @@
     <t>Registro sin nombre</t>
   </si>
   <si>
-    <t>First Name must be between 1 and 32 characters</t>
-  </si>
-  <si>
     <t>asantostest2@gmail.com</t>
   </si>
   <si>
     <t>Registro sin Apellido</t>
   </si>
   <si>
-    <t>Last Name must be between 1 and 32 characters</t>
-  </si>
-  <si>
     <t>Maria</t>
   </si>
   <si>
@@ -105,9 +99,6 @@
     <t>Registro sin Email</t>
   </si>
   <si>
-    <t>E-Mail Address does not appear to be valid</t>
-  </si>
-  <si>
     <t>Christian</t>
   </si>
   <si>
@@ -120,9 +111,6 @@
     <t>Registro sin telefono</t>
   </si>
   <si>
-    <t>Telephone must be between 3 and 32 characters</t>
-  </si>
-  <si>
     <t>Lucia</t>
   </si>
   <si>
@@ -135,9 +123,6 @@
     <t>Registro sin password</t>
   </si>
   <si>
-    <t>Password must be between 4 and 20 characters</t>
-  </si>
-  <si>
     <t>Ronald</t>
   </si>
   <si>
@@ -162,9 +147,6 @@
     <t>Password no coinciden</t>
   </si>
   <si>
-    <t>Password confirmation does not match password</t>
-  </si>
-  <si>
     <t>Oscar</t>
   </si>
   <si>
@@ -174,13 +156,31 @@
     <t>Registro con Email unico</t>
   </si>
   <si>
-    <t>Warning: E-Mail Address is already registered</t>
-  </si>
-  <si>
     <t>asantostest20@gmail.com</t>
   </si>
   <si>
     <t>asantostest1224@gmail.com</t>
+  </si>
+  <si>
+    <t>Last Name must be between 1 and 32 characters!</t>
+  </si>
+  <si>
+    <t>First Name must be between 1 and 32 characters!</t>
+  </si>
+  <si>
+    <t>Telephone must be between 3 and 32 characters!</t>
+  </si>
+  <si>
+    <t>Password must be between 4 and 20 characters!</t>
+  </si>
+  <si>
+    <t>Warning: E-Mail Address is already registered!</t>
+  </si>
+  <si>
+    <t>Password confirmation does not match password!</t>
+  </si>
+  <si>
+    <t>E-Mail Address does not appear to be valid!</t>
   </si>
 </sst>
 </file>
@@ -603,7 +603,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D2">
         <v>987654099</v>
@@ -641,7 +641,7 @@
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -649,7 +649,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4">
         <v>908765456</v>
@@ -661,18 +661,18 @@
         <v>123456</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H4" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5">
@@ -685,64 +685,64 @@
         <v>123456</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6">
+        <v>123456</v>
+      </c>
+      <c r="F6">
+        <v>123456</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6">
-        <v>123456</v>
-      </c>
-      <c r="F6">
-        <v>123456</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="H6" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D7">
         <v>986543334</v>
       </c>
       <c r="G7" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H7" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D8">
         <v>908766668</v>
@@ -754,21 +754,21 @@
         <v>123456</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H8" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D9">
         <v>908765116</v>
@@ -780,21 +780,21 @@
         <v>7890123</v>
       </c>
       <c r="G9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="D10">
         <v>900008765</v>
@@ -806,7 +806,7 @@
         <v>123456</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="H10" t="s">
         <v>46</v>

</xml_diff>